<commit_message>
Update Entity Excel files for better OS compatibility. Fix missing Peru data in Entity files.
</commit_message>
<xml_diff>
--- a/starter_pack_el_salvador/data/entity_files_calibrated/El_Salvador_Entity_Drought_Maize_calibrated.xlsx
+++ b/starter_pack_el_salvador/data/entity_files_calibrated/El_Salvador_Entity_Drought_Maize_calibrated.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30203"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30219"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fairless\OneDrive\Projects\UNU\idb\starter_packs\starter_pack_el_salvador\data\entity_files_uncalibrated\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D5ACE2C-00F9-4648-AD46-1425073D7D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{03525938-129C-4803-83C8-077F28E7840B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="10908" firstSheet="1" xr2:uid="{F478693C-5678-8847-9700-FFC3DBD3B213}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="10908" xr2:uid="{F478693C-5678-8847-9700-FFC3DBD3B213}"/>
   </bookViews>
   <sheets>
     <sheet name="assets" sheetId="1" r:id="rId1"/>
@@ -189,10 +189,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.000%"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -361,7 +362,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1"/>
@@ -390,6 +390,7 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Comma 2" xfId="7" xr:uid="{3D4C8C02-374D-E74E-9EC2-8584226DAFDD}"/>
@@ -716,571 +717,599 @@
   <dimension ref="A1:M15"/>
   <sheetFormatPr defaultColWidth="10.75" defaultRowHeight="13.15"/>
   <cols>
-    <col min="1" max="1" width="11.875" style="9" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.75" style="9"/>
-    <col min="3" max="4" width="10.875" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.25" style="9" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="13.25" style="9" customWidth="1"/>
-    <col min="10" max="13" width="10.75" style="16"/>
-    <col min="14" max="16384" width="10.75" style="9"/>
+    <col min="1" max="1" width="11.875" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.75" style="8"/>
+    <col min="3" max="4" width="10.875" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.25" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="13.25" style="8" customWidth="1"/>
+    <col min="10" max="13" width="10.75" style="15"/>
+    <col min="14" max="16384" width="10.75" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="26.45">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="25" t="s">
+      <c r="B1" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="25" t="s">
+      <c r="D1" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="25" t="s">
+      <c r="E1" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="25" t="s">
+      <c r="F1" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="25" t="s">
+      <c r="G1" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="25" t="s">
+      <c r="H1" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="25" t="s">
+      <c r="I1" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="26" t="s">
+      <c r="J1" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="26" t="s">
+      <c r="K1" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="26" t="s">
+      <c r="L1" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="26" t="s">
+      <c r="M1" s="25" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" s="9">
-        <v>1</v>
-      </c>
-      <c r="B2" s="9">
-        <v>1</v>
-      </c>
-      <c r="C2" s="9">
+      <c r="A2" s="8">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8">
+        <v>1</v>
+      </c>
+      <c r="C2" s="8">
         <v>-89.901961729999996</v>
       </c>
-      <c r="D2" s="9">
+      <c r="D2" s="8">
         <v>13.857506369999999</v>
       </c>
-      <c r="E2" s="11">
+      <c r="E2" s="10">
         <v>114614750</v>
       </c>
-      <c r="F2" s="11">
+      <c r="F2" s="10">
         <v>70252722.835613504</v>
       </c>
-      <c r="G2" s="11">
+      <c r="G2" s="10">
         <v>34227.9</v>
       </c>
-      <c r="H2" s="11">
+      <c r="H2" s="10">
         <v>114614750</v>
       </c>
-      <c r="I2" s="11">
+      <c r="I2" s="10">
         <v>3348.5767458710584</v>
       </c>
-      <c r="J2" s="8"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="8">
+      <c r="J2" s="7">
+        <v>0</v>
+      </c>
+      <c r="K2" s="14"/>
+      <c r="L2" s="7">
         <v>101</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="M2" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:13">
-      <c r="A3" s="9">
-        <v>1</v>
-      </c>
-      <c r="B3" s="9">
-        <v>1</v>
-      </c>
-      <c r="C3" s="9">
+      <c r="A3" s="8">
+        <v>1</v>
+      </c>
+      <c r="B3" s="8">
+        <v>1</v>
+      </c>
+      <c r="C3" s="8">
         <v>-88.708861069999998</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="8">
         <v>13.87704293</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="10">
         <v>48487910</v>
       </c>
-      <c r="F3" s="11">
+      <c r="F3" s="10">
         <v>35320107.099827491</v>
       </c>
-      <c r="G3" s="11">
+      <c r="G3" s="10">
         <v>15638.699999999999</v>
       </c>
-      <c r="H3" s="11">
+      <c r="H3" s="10">
         <v>48487910</v>
       </c>
-      <c r="I3" s="11">
+      <c r="I3" s="10">
         <v>3100.5077148356322</v>
       </c>
-      <c r="J3" s="8"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="8">
+      <c r="J3" s="7">
+        <v>0</v>
+      </c>
+      <c r="K3" s="14"/>
+      <c r="L3" s="7">
         <v>101</v>
       </c>
-      <c r="M3" s="8" t="s">
+      <c r="M3" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:13">
-      <c r="A4" s="9">
-        <v>1</v>
-      </c>
-      <c r="B4" s="9">
-        <v>1</v>
-      </c>
-      <c r="C4" s="9">
+      <c r="A4" s="8">
+        <v>1</v>
+      </c>
+      <c r="B4" s="8">
+        <v>1</v>
+      </c>
+      <c r="C4" s="8">
         <v>-89.074573079999993</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="8">
         <v>14.131201069999999</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="10">
         <v>58267188</v>
       </c>
-      <c r="F4" s="11">
+      <c r="F4" s="10">
         <v>18064011.111772306</v>
       </c>
-      <c r="G4" s="11">
+      <c r="G4" s="10">
         <v>19657.399999999998</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H4" s="10">
         <v>58267188</v>
       </c>
-      <c r="I4" s="11">
+      <c r="I4" s="10">
         <v>2964.1350331172998</v>
       </c>
-      <c r="J4" s="8"/>
-      <c r="K4" s="15"/>
-      <c r="L4" s="8">
+      <c r="J4" s="7">
+        <v>0</v>
+      </c>
+      <c r="K4" s="14"/>
+      <c r="L4" s="7">
         <v>101</v>
       </c>
-      <c r="M4" s="8" t="s">
+      <c r="M4" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:13">
-      <c r="A5" s="9">
-        <v>1</v>
-      </c>
-      <c r="B5" s="9">
-        <v>1</v>
-      </c>
-      <c r="C5" s="9">
+      <c r="A5" s="8">
+        <v>1</v>
+      </c>
+      <c r="B5" s="8">
+        <v>1</v>
+      </c>
+      <c r="C5" s="8">
         <v>-89.01997824</v>
       </c>
-      <c r="D5" s="9">
+      <c r="D5" s="8">
         <v>13.83557283</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="10">
         <v>29470774</v>
       </c>
-      <c r="F5" s="11">
+      <c r="F5" s="10">
         <v>58304043.30697117</v>
       </c>
-      <c r="G5" s="11">
+      <c r="G5" s="10">
         <v>10362.799999999999</v>
       </c>
-      <c r="H5" s="11">
+      <c r="H5" s="10">
         <v>29470774</v>
       </c>
-      <c r="I5" s="11">
+      <c r="I5" s="10">
         <v>2843.9006832130312</v>
       </c>
-      <c r="J5" s="8"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="8">
+      <c r="J5" s="7">
+        <v>0</v>
+      </c>
+      <c r="K5" s="14"/>
+      <c r="L5" s="7">
         <v>101</v>
       </c>
-      <c r="M5" s="8" t="s">
+      <c r="M5" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:13">
-      <c r="A6" s="9">
-        <v>1</v>
-      </c>
-      <c r="B6" s="9">
-        <v>1</v>
-      </c>
-      <c r="C6" s="9">
+      <c r="A6" s="8">
+        <v>1</v>
+      </c>
+      <c r="B6" s="8">
+        <v>1</v>
+      </c>
+      <c r="C6" s="8">
         <v>-89.362677009999999</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="8">
         <v>13.70412453</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="10">
         <v>73225698</v>
       </c>
-      <c r="F6" s="11">
+      <c r="F6" s="10">
         <v>44883443.588528864</v>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="10">
         <v>21501.199999999997</v>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="10">
         <v>73225698</v>
       </c>
-      <c r="I6" s="11">
+      <c r="I6" s="10">
         <v>3405.6563354603468</v>
       </c>
-      <c r="J6" s="8"/>
-      <c r="K6" s="15"/>
-      <c r="L6" s="8">
+      <c r="J6" s="7">
+        <v>0</v>
+      </c>
+      <c r="K6" s="14"/>
+      <c r="L6" s="7">
         <v>101</v>
       </c>
-      <c r="M6" s="8" t="s">
+      <c r="M6" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:13">
-      <c r="A7" s="9">
-        <v>1</v>
-      </c>
-      <c r="B7" s="9">
-        <v>1</v>
-      </c>
-      <c r="C7" s="9">
+      <c r="A7" s="8">
+        <v>1</v>
+      </c>
+      <c r="B7" s="8">
+        <v>1</v>
+      </c>
+      <c r="C7" s="8">
         <v>-88.964105959999998</v>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="8">
         <v>13.475231580000001</v>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="10">
         <v>40347106</v>
       </c>
-      <c r="F7" s="11">
+      <c r="F7" s="10">
         <v>18398692.221513432</v>
       </c>
-      <c r="G7" s="11">
+      <c r="G7" s="10">
         <v>11502.4</v>
       </c>
-      <c r="H7" s="11">
+      <c r="H7" s="10">
         <v>40347106</v>
       </c>
-      <c r="I7" s="11">
+      <c r="I7" s="10">
         <v>3507.7119557657534</v>
       </c>
-      <c r="J7" s="8"/>
-      <c r="K7" s="15"/>
-      <c r="L7" s="8">
+      <c r="J7" s="7">
+        <v>0</v>
+      </c>
+      <c r="K7" s="14"/>
+      <c r="L7" s="7">
         <v>101</v>
       </c>
-      <c r="M7" s="8" t="s">
+      <c r="M7" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:13">
-      <c r="A8" s="9">
-        <v>1</v>
-      </c>
-      <c r="B8" s="9">
-        <v>1</v>
-      </c>
-      <c r="C8" s="9">
+      <c r="A8" s="8">
+        <v>1</v>
+      </c>
+      <c r="B8" s="8">
+        <v>1</v>
+      </c>
+      <c r="C8" s="8">
         <v>-87.88945425</v>
       </c>
-      <c r="D8" s="9">
+      <c r="D8" s="8">
         <v>13.522977429999999</v>
       </c>
-      <c r="E8" s="11">
+      <c r="E8" s="10">
         <v>95120916</v>
       </c>
-      <c r="F8" s="11">
+      <c r="F8" s="10">
         <v>29379644.281871442</v>
       </c>
-      <c r="G8" s="11">
+      <c r="G8" s="10">
         <v>27416.899999999998</v>
       </c>
-      <c r="H8" s="11">
+      <c r="H8" s="10">
         <v>95120916</v>
       </c>
-      <c r="I8" s="11">
+      <c r="I8" s="10">
         <v>3469.4263757025778</v>
       </c>
-      <c r="J8" s="8"/>
-      <c r="K8" s="15"/>
-      <c r="L8" s="8">
+      <c r="J8" s="7">
+        <v>0</v>
+      </c>
+      <c r="K8" s="14"/>
+      <c r="L8" s="7">
         <v>101</v>
       </c>
-      <c r="M8" s="8" t="s">
+      <c r="M8" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:13">
-      <c r="A9" s="9">
-        <v>1</v>
-      </c>
-      <c r="B9" s="9">
-        <v>1</v>
-      </c>
-      <c r="C9" s="9">
+      <c r="A9" s="8">
+        <v>1</v>
+      </c>
+      <c r="B9" s="8">
+        <v>1</v>
+      </c>
+      <c r="C9" s="8">
         <v>-88.106738780000001</v>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="8">
         <v>13.76641888</v>
       </c>
-      <c r="E9" s="11">
+      <c r="E9" s="10">
         <v>30016794</v>
       </c>
-      <c r="F9" s="11">
+      <c r="F9" s="10">
         <v>17852149.792598352</v>
       </c>
-      <c r="G9" s="11">
+      <c r="G9" s="10">
         <v>9528.4</v>
       </c>
-      <c r="H9" s="11">
+      <c r="H9" s="10">
         <v>30016794</v>
       </c>
-      <c r="I9" s="11">
+      <c r="I9" s="10">
         <v>3150.2449519331685</v>
       </c>
-      <c r="J9" s="8"/>
-      <c r="K9" s="15"/>
-      <c r="L9" s="8">
+      <c r="J9" s="7">
+        <v>0</v>
+      </c>
+      <c r="K9" s="14"/>
+      <c r="L9" s="7">
         <v>101</v>
       </c>
-      <c r="M9" s="8" t="s">
+      <c r="M9" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:13">
-      <c r="A10" s="9">
-        <v>1</v>
-      </c>
-      <c r="B10" s="9">
-        <v>1</v>
-      </c>
-      <c r="C10" s="9">
+      <c r="A10" s="8">
+        <v>1</v>
+      </c>
+      <c r="B10" s="8">
+        <v>1</v>
+      </c>
+      <c r="C10" s="8">
         <v>-88.254573780000001</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="8">
         <v>13.535984040000001</v>
       </c>
-      <c r="E10" s="11">
+      <c r="E10" s="10">
         <v>57623464</v>
       </c>
-      <c r="F10" s="11">
+      <c r="F10" s="10">
         <v>34353620.235488288</v>
       </c>
-      <c r="G10" s="11">
+      <c r="G10" s="10">
         <v>16454.2</v>
       </c>
-      <c r="H10" s="11">
+      <c r="H10" s="10">
         <v>57623464</v>
       </c>
-      <c r="I10" s="11">
+      <c r="I10" s="10">
         <v>3502.0519988817441</v>
       </c>
-      <c r="J10" s="8"/>
-      <c r="K10" s="15"/>
-      <c r="L10" s="8">
+      <c r="J10" s="7">
+        <v>0</v>
+      </c>
+      <c r="K10" s="14"/>
+      <c r="L10" s="7">
         <v>101</v>
       </c>
-      <c r="M10" s="8" t="s">
+      <c r="M10" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:13">
-      <c r="A11" s="9">
-        <v>1</v>
-      </c>
-      <c r="B11" s="9">
-        <v>1</v>
-      </c>
-      <c r="C11" s="9">
+      <c r="A11" s="8">
+        <v>1</v>
+      </c>
+      <c r="B11" s="8">
+        <v>1</v>
+      </c>
+      <c r="C11" s="8">
         <v>-89.165405250000006</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="8">
         <v>13.76321484</v>
       </c>
-      <c r="E11" s="11">
+      <c r="E11" s="10">
         <v>35098276</v>
       </c>
-      <c r="F11" s="11">
+      <c r="F11" s="10">
         <v>24730621.975244187</v>
       </c>
-      <c r="G11" s="11">
+      <c r="G11" s="10">
         <v>9996.6999999999989</v>
       </c>
-      <c r="H11" s="11">
+      <c r="H11" s="10">
         <v>35098276</v>
       </c>
-      <c r="I11" s="11">
+      <c r="I11" s="10">
         <v>3510.9862254544005</v>
       </c>
-      <c r="J11" s="8"/>
-      <c r="K11" s="15"/>
-      <c r="L11" s="8">
+      <c r="J11" s="7">
+        <v>0</v>
+      </c>
+      <c r="K11" s="14"/>
+      <c r="L11" s="7">
         <v>101</v>
       </c>
-      <c r="M11" s="8" t="s">
+      <c r="M11" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:13">
-      <c r="A12" s="9">
-        <v>1</v>
-      </c>
-      <c r="B12" s="9">
-        <v>1</v>
-      </c>
-      <c r="C12" s="9">
+      <c r="A12" s="8">
+        <v>1</v>
+      </c>
+      <c r="B12" s="8">
+        <v>1</v>
+      </c>
+      <c r="C12" s="8">
         <v>-88.721138550000006</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="8">
         <v>13.601291700000001</v>
       </c>
-      <c r="E12" s="11">
+      <c r="E12" s="10">
         <v>73015018</v>
       </c>
-      <c r="F12" s="11">
+      <c r="F12" s="10">
         <v>21513369.403465658</v>
       </c>
-      <c r="G12" s="11">
+      <c r="G12" s="10">
         <v>24974.6</v>
       </c>
-      <c r="H12" s="11">
+      <c r="H12" s="10">
         <v>73015018</v>
       </c>
-      <c r="I12" s="11">
+      <c r="I12" s="10">
         <v>2923.5710682052968</v>
       </c>
-      <c r="J12" s="8"/>
-      <c r="K12" s="15"/>
-      <c r="L12" s="8">
+      <c r="J12" s="7">
+        <v>0</v>
+      </c>
+      <c r="K12" s="14"/>
+      <c r="L12" s="7">
         <v>101</v>
       </c>
-      <c r="M12" s="8" t="s">
+      <c r="M12" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:13">
-      <c r="A13" s="9">
-        <v>1</v>
-      </c>
-      <c r="B13" s="9">
-        <v>1</v>
-      </c>
-      <c r="C13" s="9">
+      <c r="A13" s="8">
+        <v>1</v>
+      </c>
+      <c r="B13" s="8">
+        <v>1</v>
+      </c>
+      <c r="C13" s="8">
         <v>-89.505248269999996</v>
       </c>
-      <c r="D13" s="9">
+      <c r="D13" s="8">
         <v>14.11748882</v>
       </c>
-      <c r="E13" s="11">
+      <c r="E13" s="10">
         <v>56046676</v>
       </c>
-      <c r="F13" s="11">
+      <c r="F13" s="10">
         <v>29720500.215793975</v>
       </c>
-      <c r="G13" s="11">
+      <c r="G13" s="10">
         <v>27369.3</v>
       </c>
-      <c r="H13" s="11">
+      <c r="H13" s="10">
         <v>56046676</v>
       </c>
-      <c r="I13" s="11">
+      <c r="I13" s="10">
         <v>2047.7935497071537</v>
       </c>
-      <c r="J13" s="8"/>
-      <c r="K13" s="15"/>
-      <c r="L13" s="8">
+      <c r="J13" s="7">
+        <v>0</v>
+      </c>
+      <c r="K13" s="14"/>
+      <c r="L13" s="7">
         <v>101</v>
       </c>
-      <c r="M13" s="8" t="s">
+      <c r="M13" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:13">
-      <c r="A14" s="9">
-        <v>1</v>
-      </c>
-      <c r="B14" s="9">
-        <v>1</v>
-      </c>
-      <c r="C14" s="9">
+      <c r="A14" s="8">
+        <v>1</v>
+      </c>
+      <c r="B14" s="8">
+        <v>1</v>
+      </c>
+      <c r="C14" s="8">
         <v>-89.684284340000005</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="8">
         <v>13.694153849999999</v>
       </c>
-      <c r="E14" s="11">
+      <c r="E14" s="10">
         <v>29125130</v>
       </c>
-      <c r="F14" s="11">
+      <c r="F14" s="10">
         <v>35714675.545465007</v>
       </c>
-      <c r="G14" s="11">
+      <c r="G14" s="10">
         <v>14678.999999999998</v>
       </c>
-      <c r="H14" s="11">
+      <c r="H14" s="10">
         <v>29125130</v>
       </c>
-      <c r="I14" s="11">
+      <c r="I14" s="10">
         <v>1984.135840316098</v>
       </c>
-      <c r="J14" s="8"/>
-      <c r="K14" s="15"/>
-      <c r="L14" s="8">
+      <c r="J14" s="7">
+        <v>0</v>
+      </c>
+      <c r="K14" s="14"/>
+      <c r="L14" s="7">
         <v>101</v>
       </c>
-      <c r="M14" s="8" t="s">
+      <c r="M14" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:13">
-      <c r="A15" s="9">
-        <v>1</v>
-      </c>
-      <c r="B15" s="9">
-        <v>1</v>
-      </c>
-      <c r="C15" s="9">
+      <c r="A15" s="8">
+        <v>1</v>
+      </c>
+      <c r="B15" s="8">
+        <v>1</v>
+      </c>
+      <c r="C15" s="8">
         <v>-88.490388339999996</v>
       </c>
-      <c r="D15" s="9">
+      <c r="D15" s="8">
         <v>13.382104379999999</v>
       </c>
-      <c r="E15" s="11">
+      <c r="E15" s="10">
         <v>47931816</v>
       </c>
-      <c r="F15" s="11">
+      <c r="F15" s="10">
         <v>44754307.996059246</v>
       </c>
-      <c r="G15" s="11">
+      <c r="G15" s="10">
         <v>20405</v>
       </c>
-      <c r="H15" s="11">
+      <c r="H15" s="10">
         <v>47931816</v>
       </c>
-      <c r="I15" s="11">
+      <c r="I15" s="10">
         <v>2349.0230825777994</v>
       </c>
-      <c r="J15" s="8"/>
-      <c r="K15" s="15"/>
-      <c r="L15" s="8">
+      <c r="J15" s="7">
+        <v>0</v>
+      </c>
+      <c r="K15" s="14"/>
+      <c r="L15" s="7">
         <v>101</v>
       </c>
-      <c r="M15" s="8" t="s">
+      <c r="M15" s="7" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1296,453 +1325,453 @@
   <dimension ref="A1:H82"/>
   <sheetFormatPr defaultColWidth="11.5" defaultRowHeight="12.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="11.75" style="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="11.5" style="12"/>
-    <col min="6" max="6" width="24.875" style="12" customWidth="1"/>
-    <col min="7" max="7" width="11.5" style="12"/>
-    <col min="8" max="16384" width="11.5" style="10"/>
+    <col min="1" max="1" width="11.75" style="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="11.5" style="11"/>
+    <col min="6" max="6" width="24.875" style="11" customWidth="1"/>
+    <col min="7" max="7" width="11.5" style="11"/>
+    <col min="8" max="16384" width="11.5" style="9"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="C1" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="27" t="s">
+      <c r="D1" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="27" t="s">
+      <c r="E1" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="28" t="s">
+      <c r="F1" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="G1" s="28" t="s">
+      <c r="G1" s="27" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="12">
+      <c r="A2" s="11">
         <v>101</v>
       </c>
-      <c r="B2" s="12">
+      <c r="B2" s="11">
         <v>-2.5499999999999998</v>
       </c>
-      <c r="C2" s="29">
+      <c r="C2" s="28">
         <v>0.6</v>
       </c>
-      <c r="D2" s="12">
-        <v>1</v>
-      </c>
-      <c r="E2" s="12" t="s">
+      <c r="D2" s="11">
+        <v>1</v>
+      </c>
+      <c r="E2" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G2" s="11" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="12">
+      <c r="A3" s="11">
         <v>101</v>
       </c>
-      <c r="B3" s="12">
+      <c r="B3" s="11">
         <v>-2.3290000000000002</v>
       </c>
-      <c r="C3" s="29">
+      <c r="C3" s="28">
         <v>0.441</v>
       </c>
-      <c r="D3" s="12">
-        <v>1</v>
-      </c>
-      <c r="E3" s="12" t="s">
+      <c r="D3" s="11">
+        <v>1</v>
+      </c>
+      <c r="E3" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="G3" s="12" t="s">
+      <c r="G3" s="11" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="12">
+      <c r="A4" s="11">
         <v>101</v>
       </c>
-      <c r="B4" s="12">
+      <c r="B4" s="11">
         <v>-2.1070000000000002</v>
       </c>
-      <c r="C4" s="29">
+      <c r="C4" s="28">
         <v>0.30599999999999999</v>
       </c>
-      <c r="D4" s="12">
-        <v>1</v>
-      </c>
-      <c r="E4" s="12" t="s">
+      <c r="D4" s="11">
+        <v>1</v>
+      </c>
+      <c r="E4" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="G4" s="11" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="12">
+      <c r="A5" s="11">
         <v>101</v>
       </c>
-      <c r="B5" s="12">
+      <c r="B5" s="11">
         <v>-1.8859999999999999</v>
       </c>
-      <c r="C5" s="29">
+      <c r="C5" s="28">
         <v>0.19600000000000001</v>
       </c>
-      <c r="D5" s="12">
-        <v>1</v>
-      </c>
-      <c r="E5" s="12" t="s">
+      <c r="D5" s="11">
+        <v>1</v>
+      </c>
+      <c r="E5" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="G5" s="12" t="s">
+      <c r="G5" s="11" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="12">
+      <c r="A6" s="11">
         <v>101</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="11">
         <v>-1.6639999999999999</v>
       </c>
-      <c r="C6" s="29">
+      <c r="C6" s="28">
         <v>0.11</v>
       </c>
-      <c r="D6" s="12">
-        <v>1</v>
-      </c>
-      <c r="E6" s="12" t="s">
+      <c r="D6" s="11">
+        <v>1</v>
+      </c>
+      <c r="E6" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="G6" s="12" t="s">
+      <c r="G6" s="11" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="12">
+      <c r="A7" s="11">
         <v>101</v>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="11">
         <v>-1.4430000000000001</v>
       </c>
-      <c r="C7" s="29">
+      <c r="C7" s="28">
         <v>4.9000000000000002E-2</v>
       </c>
-      <c r="D7" s="12">
-        <v>1</v>
-      </c>
-      <c r="E7" s="12" t="s">
+      <c r="D7" s="11">
+        <v>1</v>
+      </c>
+      <c r="E7" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="G7" s="12" t="s">
+      <c r="G7" s="11" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="12">
+      <c r="A8" s="11">
         <v>101</v>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="11">
         <v>-1.2210000000000001</v>
       </c>
-      <c r="C8" s="29">
+      <c r="C8" s="28">
         <v>1.2E-2</v>
       </c>
-      <c r="D8" s="12">
-        <v>1</v>
-      </c>
-      <c r="E8" s="12" t="s">
+      <c r="D8" s="11">
+        <v>1</v>
+      </c>
+      <c r="E8" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="12" t="s">
+      <c r="G8" s="11" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="12">
+      <c r="A9" s="11">
         <v>101</v>
       </c>
-      <c r="B9" s="12">
+      <c r="B9" s="11">
         <v>-1</v>
       </c>
-      <c r="C9" s="29">
+      <c r="C9" s="28">
         <v>0</v>
       </c>
-      <c r="D9" s="12">
-        <v>1</v>
-      </c>
-      <c r="E9" s="12" t="s">
+      <c r="D9" s="11">
+        <v>1</v>
+      </c>
+      <c r="E9" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="G9" s="12" t="s">
+      <c r="G9" s="11" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="15">
-      <c r="A13" s="21"/>
-      <c r="B13" s="21"/>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
-      <c r="G13" s="21"/>
-      <c r="H13" s="13"/>
+      <c r="A13" s="20"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="12"/>
     </row>
     <row r="14" spans="1:8" ht="15">
-      <c r="A14" s="21"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="21"/>
-      <c r="G14" s="22"/>
-      <c r="H14" s="13"/>
+      <c r="A14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="12"/>
     </row>
     <row r="15" spans="1:8" ht="15">
-      <c r="A15" s="21"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="13"/>
+      <c r="A15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="21"/>
+      <c r="H15" s="12"/>
     </row>
     <row r="16" spans="1:8" ht="15">
-      <c r="A16" s="21"/>
-      <c r="B16" s="21"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="13"/>
+      <c r="A16" s="20"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="21"/>
+      <c r="H16" s="12"/>
     </row>
     <row r="17" spans="1:8" ht="15">
-      <c r="A17" s="21"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
-      <c r="F17" s="21"/>
-      <c r="G17" s="22"/>
-      <c r="H17" s="13"/>
+      <c r="A17" s="20"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="21"/>
+      <c r="H17" s="12"/>
     </row>
     <row r="18" spans="1:8" ht="15">
-      <c r="A18" s="21"/>
-      <c r="B18" s="21"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="13"/>
+      <c r="A18" s="20"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="20"/>
+      <c r="G18" s="21"/>
+      <c r="H18" s="12"/>
     </row>
     <row r="19" spans="1:8" ht="15">
-      <c r="A19" s="21"/>
-      <c r="B19" s="21"/>
-      <c r="C19" s="21"/>
-      <c r="D19" s="21"/>
-      <c r="E19" s="21"/>
-      <c r="F19" s="21"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="13"/>
+      <c r="A19" s="20"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="21"/>
+      <c r="H19" s="12"/>
     </row>
     <row r="20" spans="1:8" ht="15">
-      <c r="A20" s="21"/>
-      <c r="B20" s="21"/>
-      <c r="C20" s="21"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="21"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="13"/>
+      <c r="A20" s="20"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="21"/>
+      <c r="H20" s="12"/>
     </row>
     <row r="21" spans="1:8" ht="15">
-      <c r="A21" s="21"/>
-      <c r="B21" s="21"/>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="13"/>
+      <c r="A21" s="20"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="21"/>
+      <c r="H21" s="12"/>
     </row>
     <row r="22" spans="1:8" ht="15">
-      <c r="A22" s="21"/>
-      <c r="B22" s="21"/>
-      <c r="C22" s="21"/>
-      <c r="D22" s="21"/>
-      <c r="E22" s="21"/>
-      <c r="F22" s="21"/>
-      <c r="G22" s="22"/>
-      <c r="H22" s="13"/>
+      <c r="A22" s="20"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="21"/>
+      <c r="H22" s="12"/>
     </row>
     <row r="23" spans="1:8" ht="15">
-      <c r="A23" s="21"/>
-      <c r="B23" s="21"/>
-      <c r="C23" s="21"/>
-      <c r="D23" s="21"/>
-      <c r="E23" s="21"/>
-      <c r="F23" s="21"/>
-      <c r="G23" s="22"/>
-      <c r="H23" s="13"/>
+      <c r="A23" s="20"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="20"/>
+      <c r="G23" s="21"/>
+      <c r="H23" s="12"/>
     </row>
     <row r="24" spans="1:8" ht="15">
-      <c r="A24" s="21"/>
-      <c r="B24" s="21"/>
-      <c r="C24" s="21"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="21"/>
-      <c r="F24" s="21"/>
-      <c r="G24" s="22"/>
-      <c r="H24" s="13"/>
+      <c r="A24" s="20"/>
+      <c r="B24" s="20"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="21"/>
+      <c r="H24" s="12"/>
     </row>
     <row r="25" spans="1:8" ht="15">
-      <c r="A25" s="21"/>
-      <c r="B25" s="21"/>
-      <c r="C25" s="21"/>
-      <c r="D25" s="21"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
-      <c r="G25" s="22"/>
-      <c r="H25" s="13"/>
+      <c r="A25" s="20"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="21"/>
+      <c r="H25" s="12"/>
     </row>
     <row r="56" spans="1:6">
-      <c r="A56" s="23"/>
-      <c r="F56" s="23"/>
+      <c r="A56" s="22"/>
+      <c r="F56" s="22"/>
     </row>
     <row r="57" spans="1:6">
-      <c r="A57" s="23"/>
-      <c r="F57" s="23"/>
+      <c r="A57" s="22"/>
+      <c r="F57" s="22"/>
     </row>
     <row r="58" spans="1:6">
-      <c r="A58" s="23"/>
-      <c r="F58" s="23"/>
+      <c r="A58" s="22"/>
+      <c r="F58" s="22"/>
     </row>
     <row r="59" spans="1:6">
-      <c r="A59" s="23"/>
-      <c r="F59" s="23"/>
+      <c r="A59" s="22"/>
+      <c r="F59" s="22"/>
     </row>
     <row r="60" spans="1:6">
-      <c r="A60" s="23"/>
-      <c r="F60" s="23"/>
+      <c r="A60" s="22"/>
+      <c r="F60" s="22"/>
     </row>
     <row r="61" spans="1:6">
-      <c r="A61" s="23"/>
-      <c r="F61" s="23"/>
+      <c r="A61" s="22"/>
+      <c r="F61" s="22"/>
     </row>
     <row r="62" spans="1:6">
-      <c r="A62" s="23"/>
-      <c r="F62" s="23"/>
+      <c r="A62" s="22"/>
+      <c r="F62" s="22"/>
     </row>
     <row r="63" spans="1:6">
-      <c r="A63" s="23"/>
-      <c r="F63" s="23"/>
+      <c r="A63" s="22"/>
+      <c r="F63" s="22"/>
     </row>
     <row r="64" spans="1:6">
-      <c r="A64" s="23"/>
-      <c r="F64" s="23"/>
+      <c r="A64" s="22"/>
+      <c r="F64" s="22"/>
     </row>
     <row r="65" spans="1:6">
-      <c r="A65" s="23"/>
-      <c r="F65" s="23"/>
+      <c r="A65" s="22"/>
+      <c r="F65" s="22"/>
     </row>
     <row r="66" spans="1:6">
-      <c r="A66" s="23"/>
-      <c r="F66" s="23"/>
+      <c r="A66" s="22"/>
+      <c r="F66" s="22"/>
     </row>
     <row r="67" spans="1:6">
-      <c r="A67" s="23"/>
-      <c r="F67" s="23"/>
+      <c r="A67" s="22"/>
+      <c r="F67" s="22"/>
     </row>
     <row r="68" spans="1:6">
-      <c r="A68" s="23"/>
-      <c r="F68" s="23"/>
+      <c r="A68" s="22"/>
+      <c r="F68" s="22"/>
     </row>
     <row r="69" spans="1:6">
-      <c r="A69" s="23"/>
-      <c r="F69" s="23"/>
+      <c r="A69" s="22"/>
+      <c r="F69" s="22"/>
     </row>
     <row r="70" spans="1:6">
-      <c r="A70" s="23"/>
-      <c r="F70" s="23"/>
+      <c r="A70" s="22"/>
+      <c r="F70" s="22"/>
     </row>
     <row r="71" spans="1:6">
-      <c r="A71" s="23"/>
-      <c r="F71" s="23"/>
+      <c r="A71" s="22"/>
+      <c r="F71" s="22"/>
     </row>
     <row r="72" spans="1:6">
-      <c r="A72" s="23"/>
-      <c r="F72" s="23"/>
+      <c r="A72" s="22"/>
+      <c r="F72" s="22"/>
     </row>
     <row r="73" spans="1:6">
-      <c r="A73" s="23"/>
-      <c r="F73" s="23"/>
+      <c r="A73" s="22"/>
+      <c r="F73" s="22"/>
     </row>
     <row r="74" spans="1:6">
-      <c r="A74" s="23"/>
-      <c r="F74" s="23"/>
+      <c r="A74" s="22"/>
+      <c r="F74" s="22"/>
     </row>
     <row r="75" spans="1:6">
-      <c r="A75" s="23"/>
-      <c r="F75" s="23"/>
+      <c r="A75" s="22"/>
+      <c r="F75" s="22"/>
     </row>
     <row r="76" spans="1:6">
-      <c r="A76" s="23"/>
-      <c r="F76" s="23"/>
+      <c r="A76" s="22"/>
+      <c r="F76" s="22"/>
     </row>
     <row r="77" spans="1:6">
-      <c r="A77" s="23"/>
-      <c r="F77" s="23"/>
+      <c r="A77" s="22"/>
+      <c r="F77" s="22"/>
     </row>
     <row r="78" spans="1:6">
-      <c r="A78" s="23"/>
-      <c r="F78" s="23"/>
+      <c r="A78" s="22"/>
+      <c r="F78" s="22"/>
     </row>
     <row r="79" spans="1:6">
-      <c r="A79" s="23"/>
-      <c r="F79" s="23"/>
+      <c r="A79" s="22"/>
+      <c r="F79" s="22"/>
     </row>
     <row r="80" spans="1:6">
-      <c r="A80" s="23"/>
-      <c r="F80" s="23"/>
+      <c r="A80" s="22"/>
+      <c r="F80" s="22"/>
     </row>
     <row r="81" spans="1:6">
-      <c r="A81" s="23"/>
-      <c r="F81" s="23"/>
+      <c r="A81" s="22"/>
+      <c r="F81" s="22"/>
     </row>
     <row r="82" spans="1:6">
-      <c r="A82" s="23"/>
-      <c r="F82" s="23"/>
+      <c r="A82" s="22"/>
+      <c r="F82" s="22"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -1760,219 +1789,219 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="19" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" ht="12.75">
       <c r="A2" s="6">
         <v>2025</v>
       </c>
-      <c r="B2" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
+      <c r="B2" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="12.75">
       <c r="A3" s="6">
         <v>2026</v>
       </c>
-      <c r="B3" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
+      <c r="B3" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="12.75">
       <c r="A4" s="6">
         <v>2027</v>
       </c>
-      <c r="B4" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
+      <c r="B4" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="12.75">
       <c r="A5" s="6">
         <v>2028</v>
       </c>
-      <c r="B5" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
+      <c r="B5" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="12.75">
       <c r="A6" s="6">
         <v>2029</v>
       </c>
-      <c r="B6" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
+      <c r="B6" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="12.75">
       <c r="A7" s="6">
         <v>2030</v>
       </c>
-      <c r="B7" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
+      <c r="B7" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="12.75">
       <c r="A8" s="6">
         <v>2031</v>
       </c>
-      <c r="B8" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
+      <c r="B8" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="12.75">
       <c r="A9" s="6">
         <v>2032</v>
       </c>
-      <c r="B9" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2">
+      <c r="B9" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="12.75">
       <c r="A10" s="6">
         <v>2033</v>
       </c>
-      <c r="B10" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2">
+      <c r="B10" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="12.75">
       <c r="A11" s="6">
         <v>2034</v>
       </c>
-      <c r="B11" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2">
+      <c r="B11" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="12.75">
       <c r="A12" s="6">
         <v>2035</v>
       </c>
-      <c r="B12" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2">
+      <c r="B12" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="12.75">
       <c r="A13" s="6">
         <v>2036</v>
       </c>
-      <c r="B13" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2">
+      <c r="B13" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="12.75">
       <c r="A14" s="6">
         <v>2037</v>
       </c>
-      <c r="B14" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2">
+      <c r="B14" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="12.75">
       <c r="A15" s="6">
         <v>2038</v>
       </c>
-      <c r="B15" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2">
+      <c r="B15" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="12.75">
       <c r="A16" s="6">
         <v>2039</v>
       </c>
-      <c r="B16" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2">
+      <c r="B16" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="12.75">
       <c r="A17" s="6">
         <v>2040</v>
       </c>
-      <c r="B17" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
+      <c r="B17" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="12.75">
       <c r="A18" s="6">
         <v>2041</v>
       </c>
-      <c r="B18" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2">
+      <c r="B18" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="12.75">
       <c r="A19" s="6">
         <v>2042</v>
       </c>
-      <c r="B19" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2">
+      <c r="B19" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="12.75">
       <c r="A20" s="6">
         <v>2043</v>
       </c>
-      <c r="B20" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2">
+      <c r="B20" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="12.75">
       <c r="A21" s="6">
         <v>2044</v>
       </c>
-      <c r="B21" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2">
+      <c r="B21" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="12.75">
       <c r="A22" s="6">
         <v>2045</v>
       </c>
-      <c r="B22" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2">
+      <c r="B22" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="12.75">
       <c r="A23" s="6">
         <v>2046</v>
       </c>
-      <c r="B23" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2">
+      <c r="B23" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="12.75">
       <c r="A24" s="6">
         <v>2047</v>
       </c>
-      <c r="B24" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2">
+      <c r="B24" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="12.75">
       <c r="A25" s="6">
         <v>2048</v>
       </c>
-      <c r="B25" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2">
+      <c r="B25" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="12.75">
       <c r="A26" s="6">
         <v>2049</v>
       </c>
-      <c r="B26" s="7">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2">
+      <c r="B26" s="29">
+        <v>1.3999999999999999E-4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="12.75">
       <c r="A27" s="6">
         <v>2050</v>
       </c>
-      <c r="B27" s="7">
-        <v>0.02</v>
+      <c r="B27" s="29">
+        <v>1.3999999999999999E-4</v>
       </c>
     </row>
   </sheetData>
@@ -1998,93 +2027,93 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" s="5" customFormat="1" ht="39.6">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="F1" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="G1" s="18" t="s">
+      <c r="G1" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="H1" s="18" t="s">
+      <c r="H1" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="I1" s="18" t="s">
+      <c r="I1" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="J1" s="18" t="s">
+      <c r="J1" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="K1" s="18" t="s">
+      <c r="K1" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="L1" s="18" t="s">
+      <c r="L1" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="M1" s="17" t="s">
+      <c r="M1" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="N1" s="17" t="s">
+      <c r="N1" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="O1" s="18" t="s">
+      <c r="O1" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="P1" s="18" t="s">
+      <c r="P1" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="Q1" s="18" t="s">
+      <c r="Q1" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="R1" s="17" t="s">
+      <c r="R1" s="16" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="13.15">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="14">
+      <c r="C2" s="13">
         <v>0</v>
       </c>
-      <c r="D2" s="14">
-        <v>1</v>
-      </c>
-      <c r="E2" s="14">
+      <c r="D2" s="13">
+        <v>1</v>
+      </c>
+      <c r="E2" s="13">
         <v>0</v>
       </c>
-      <c r="F2" s="14">
+      <c r="F2" s="13">
         <v>0</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="H2" s="14">
-        <v>1</v>
-      </c>
-      <c r="I2" s="14">
+      <c r="H2" s="13">
+        <v>1</v>
+      </c>
+      <c r="I2" s="13">
         <v>0</v>
       </c>
-      <c r="J2" s="14">
-        <v>1</v>
-      </c>
-      <c r="K2" s="14">
+      <c r="J2" s="13">
+        <v>1</v>
+      </c>
+      <c r="K2" s="13">
         <v>0</v>
       </c>
       <c r="L2" s="2" t="s">
@@ -2110,95 +2139,95 @@
       </c>
     </row>
     <row r="3" spans="1:18" ht="13.15">
-      <c r="A3" s="14"/>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
     </row>
     <row r="4" spans="1:18" ht="13.15">
-      <c r="A4" s="14"/>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="14"/>
-      <c r="K4" s="14"/>
+      <c r="A4" s="13"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
+      <c r="I4" s="13"/>
+      <c r="J4" s="13"/>
+      <c r="K4" s="13"/>
     </row>
     <row r="5" spans="1:18" ht="13.15">
-      <c r="A5" s="14"/>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
+      <c r="A5" s="13"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
+      <c r="I5" s="13"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="13"/>
     </row>
     <row r="6" spans="1:18" ht="13.15">
-      <c r="A6" s="14"/>
-      <c r="B6" s="14"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="14"/>
-      <c r="J6" s="14"/>
-      <c r="K6" s="14"/>
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
+      <c r="I6" s="13"/>
+      <c r="J6" s="13"/>
+      <c r="K6" s="13"/>
     </row>
     <row r="7" spans="1:18" s="4" customFormat="1" ht="13.15">
-      <c r="A7" s="14"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="14"/>
-      <c r="J7" s="14"/>
-      <c r="K7" s="14"/>
+      <c r="A7" s="13"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
     </row>
     <row r="8" spans="1:18" ht="13.15">
-      <c r="A8" s="14"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="14"/>
+      <c r="A8" s="13"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
+      <c r="I8" s="13"/>
+      <c r="J8" s="13"/>
+      <c r="K8" s="13"/>
     </row>
     <row r="9" spans="1:18" ht="13.15">
-      <c r="A9" s="14"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="14"/>
-      <c r="J9" s="14"/>
-      <c r="K9" s="14"/>
+      <c r="A9" s="13"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="13"/>
+      <c r="I9" s="13"/>
+      <c r="J9" s="13"/>
+      <c r="K9" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2208,6 +2237,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005635FBEDCBF528448E90466BDCE740AC" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d906b7f2ac9a894dfa93f76c288966b0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="fec4f95d-6d6e-4554-9489-9adf9faabb3f" xmlns:ns3="85675493-fe14-4357-9e44-2c2e96e19a02" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c38a7734914d84977eedbcf1df588f4c" ns2:_="" ns3:_="">
     <xsd:import namespace="fec4f95d-6d6e-4554-9489-9adf9faabb3f"/>
@@ -2456,15 +2494,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2477,11 +2506,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E35089F5-58B8-4A47-B7DC-A0680923C4F3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B725CAAD-7610-4431-B145-B83D84FEBFE9}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B725CAAD-7610-4431-B145-B83D84FEBFE9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E35089F5-58B8-4A47-B7DC-A0680923C4F3}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
El Salvador: Correction: production units are kg not USD!
</commit_message>
<xml_diff>
--- a/starter_pack_el_salvador/data/entity_files_calibrated/El_Salvador_Entity_Drought_Maize_calibrated.xlsx
+++ b/starter_pack_el_salvador/data/entity_files_calibrated/El_Salvador_Entity_Drought_Maize_calibrated.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30219"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30224"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fairless\OneDrive\Projects\UNU\idb\starter_packs\starter_pack_el_salvador\data\entity_files_uncalibrated\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{03525938-129C-4803-83C8-077F28E7840B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9E7FC5AD-42ED-47E1-AE5A-6A693EDA17DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="10908" xr2:uid="{F478693C-5678-8847-9700-FFC3DBD3B213}"/>
   </bookViews>
@@ -83,7 +83,7 @@
     <t>Value_unit</t>
   </si>
   <si>
-    <t>USD</t>
+    <t>kg</t>
   </si>
   <si>
     <t>impact_fun_id</t>
@@ -2237,15 +2237,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005635FBEDCBF528448E90466BDCE740AC" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d906b7f2ac9a894dfa93f76c288966b0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="fec4f95d-6d6e-4554-9489-9adf9faabb3f" xmlns:ns3="85675493-fe14-4357-9e44-2c2e96e19a02" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c38a7734914d84977eedbcf1df588f4c" ns2:_="" ns3:_="">
     <xsd:import namespace="fec4f95d-6d6e-4554-9489-9adf9faabb3f"/>
@@ -2494,7 +2485,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="85675493-fe14-4357-9e44-2c2e96e19a02" xsi:nil="true"/>
@@ -2505,14 +2496,23 @@
 </p:properties>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B725CAAD-7610-4431-B145-B83D84FEBFE9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E35089F5-58B8-4A47-B7DC-A0680923C4F3}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E35089F5-58B8-4A47-B7DC-A0680923C4F3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{87E1C1E2-1870-4C84-B3FA-2AAA1CA77D14}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{87E1C1E2-1870-4C84-B3FA-2AAA1CA77D14}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B725CAAD-7610-4431-B145-B83D84FEBFE9}"/>
 </file>
</xml_diff>